<commit_message>
Committing delete employee module test cases
</commit_message>
<xml_diff>
--- a/UIHRMAutomationFramework/src/test/resources/TestData.xlsx
+++ b/UIHRMAutomationFramework/src/test/resources/TestData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/bec74d40107829ab/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="198" documentId="8_{D6872387-AE08-4DF3-8870-05A84F213211}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{33F34819-56C9-4F5A-A66A-7C8B80D6BD39}"/>
+  <xr:revisionPtr revIDLastSave="242" documentId="8_{D6872387-AE08-4DF3-8870-05A84F213211}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5027C546-B57C-4328-AA76-0C2A3905CFBE}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="4" xr2:uid="{C6793B7E-5E58-4769-A8F2-79D9A112E6E1}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="5" xr2:uid="{C6793B7E-5E58-4769-A8F2-79D9A112E6E1}"/>
   </bookViews>
   <sheets>
     <sheet name="Login" sheetId="1" r:id="rId1"/>
@@ -18,6 +18,7 @@
     <sheet name="AddEmployee" sheetId="3" r:id="rId3"/>
     <sheet name="SearchEmployee" sheetId="4" r:id="rId4"/>
     <sheet name="UpdateEmployee" sheetId="5" r:id="rId5"/>
+    <sheet name="DeleteEmployee" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="207" uniqueCount="82">
   <si>
     <t>Username</t>
   </si>
@@ -256,6 +257,36 @@
   </si>
   <si>
     <t>TC31</t>
+  </si>
+  <si>
+    <t>TC32</t>
+  </si>
+  <si>
+    <t>TC33</t>
+  </si>
+  <si>
+    <t>0295</t>
+  </si>
+  <si>
+    <t>TC34</t>
+  </si>
+  <si>
+    <t>TC35</t>
+  </si>
+  <si>
+    <t>TC36</t>
+  </si>
+  <si>
+    <t>TC37</t>
+  </si>
+  <si>
+    <t>TC38</t>
+  </si>
+  <si>
+    <t>TC39</t>
+  </si>
+  <si>
+    <t>01715</t>
   </si>
 </sst>
 </file>
@@ -1336,4 +1367,199 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F7F7F8F1-999E-455A-9FCF-D518EFF7A1AE}">
+  <dimension ref="A1:E21"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="10.109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>72</v>
+      </c>
+      <c r="B2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C2" t="s">
+        <v>3</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="E2" s="1"/>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>73</v>
+      </c>
+      <c r="B3" t="s">
+        <v>2</v>
+      </c>
+      <c r="C3" t="s">
+        <v>3</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="E3" s="1"/>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>75</v>
+      </c>
+      <c r="B4" t="s">
+        <v>2</v>
+      </c>
+      <c r="C4" t="s">
+        <v>3</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="E4" s="1"/>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>76</v>
+      </c>
+      <c r="B5" t="s">
+        <v>2</v>
+      </c>
+      <c r="C5" t="s">
+        <v>3</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="E5" s="1"/>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>77</v>
+      </c>
+      <c r="B6" t="s">
+        <v>2</v>
+      </c>
+      <c r="C6" t="s">
+        <v>3</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="E6" s="1"/>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B7" t="s">
+        <v>2</v>
+      </c>
+      <c r="C7" t="s">
+        <v>3</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="E7" s="1"/>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>79</v>
+      </c>
+      <c r="B8" t="s">
+        <v>2</v>
+      </c>
+      <c r="C8" t="s">
+        <v>3</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="E8" s="1"/>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>80</v>
+      </c>
+      <c r="B9" t="s">
+        <v>2</v>
+      </c>
+      <c r="C9" t="s">
+        <v>3</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="E9" s="1"/>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="D10" s="1"/>
+      <c r="E10" s="1"/>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="D11" s="1"/>
+      <c r="E11" s="1"/>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="D12" s="1"/>
+      <c r="E12" s="1"/>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="D13" s="1"/>
+      <c r="E13" s="1"/>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="D14" s="1"/>
+      <c r="E14" s="1"/>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="D15" s="1"/>
+      <c r="E15" s="1"/>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="D16" s="1"/>
+      <c r="E16" s="1"/>
+    </row>
+    <row r="17" spans="4:5" x14ac:dyDescent="0.3">
+      <c r="D17" s="1"/>
+      <c r="E17" s="1"/>
+    </row>
+    <row r="18" spans="4:5" x14ac:dyDescent="0.3">
+      <c r="D18" s="1"/>
+      <c r="E18" s="1"/>
+    </row>
+    <row r="19" spans="4:5" x14ac:dyDescent="0.3">
+      <c r="D19" s="1"/>
+      <c r="E19" s="1"/>
+    </row>
+    <row r="20" spans="4:5" x14ac:dyDescent="0.3">
+      <c r="D20" s="1"/>
+      <c r="E20" s="1"/>
+    </row>
+    <row r="21" spans="4:5" x14ac:dyDescent="0.3">
+      <c r="D21" s="1"/>
+      <c r="E21" s="1"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>